<commit_message>
Final Draft for College Pre-Submission Review
Final draft and minor Associate Dean edits incorporated
</commit_message>
<xml_diff>
--- a/Scholarly_Activity/scholarly_activity_chart.xlsx
+++ b/Scholarly_Activity/scholarly_activity_chart.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dcham\Documents\GitHub\Chamberlain_Tenure_Packet\Scholarly_Activity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D7DF954-AD66-4093-9453-05D21B430124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB093087-2EE7-4CF6-ABAF-E1F5A6924ACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4470" yWindow="735" windowWidth="42255" windowHeight="20280" xr2:uid="{7E679648-1FC1-4A4C-BFC2-A85F22ED829C}"/>
+    <workbookView xWindow="1500" yWindow="1230" windowWidth="47235" windowHeight="20280" xr2:uid="{7E679648-1FC1-4A4C-BFC2-A85F22ED829C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -132,7 +132,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="22"/>
+      <sz val="36"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -140,7 +140,7 @@
     </font>
     <font>
       <b/>
-      <sz val="22"/>
+      <sz val="36"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -489,7 +489,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -619,6 +619,7 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -953,27 +954,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D602E43B-B0A2-4EA1-BB6D-602EBF400D0A}">
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:P14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="1"/>
-    <col min="2" max="2" width="30.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" customWidth="1"/>
-    <col min="5" max="5" width="23.42578125" customWidth="1"/>
-    <col min="6" max="6" width="24.28515625" customWidth="1"/>
-    <col min="7" max="7" width="21.85546875" customWidth="1"/>
-    <col min="8" max="8" width="23" customWidth="1"/>
-    <col min="9" max="9" width="23.140625" customWidth="1"/>
-    <col min="10" max="10" width="13.28515625" customWidth="1"/>
-    <col min="11" max="11" width="15.85546875" customWidth="1"/>
-    <col min="12" max="12" width="18.7109375" customWidth="1"/>
-    <col min="13" max="13" width="15.42578125" customWidth="1"/>
-    <col min="14" max="14" width="18.7109375" customWidth="1"/>
+    <col min="1" max="1" width="3.85546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="49.140625" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="4" max="4" width="24.140625" customWidth="1"/>
+    <col min="5" max="5" width="36.85546875" customWidth="1"/>
+    <col min="6" max="6" width="39.42578125" customWidth="1"/>
+    <col min="7" max="7" width="35.28515625" customWidth="1"/>
+    <col min="8" max="8" width="35.5703125" customWidth="1"/>
+    <col min="9" max="9" width="36.7109375" customWidth="1"/>
+    <col min="10" max="10" width="22.28515625" customWidth="1"/>
+    <col min="11" max="11" width="25.140625" customWidth="1"/>
+    <col min="12" max="12" width="29.5703125" customWidth="1"/>
+    <col min="13" max="13" width="24" customWidth="1"/>
+    <col min="14" max="14" width="30.140625" customWidth="1"/>
     <col min="15" max="15" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:16" s="1" customFormat="1" ht="29.25" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="1" spans="2:16" s="1" customFormat="1" ht="47.25" thickBot="1" x14ac:dyDescent="0.75">
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
@@ -987,8 +988,9 @@
       <c r="L1" s="2"/>
       <c r="M1" s="2"/>
       <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
     </row>
-    <row r="2" spans="2:16" ht="29.25" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="2" spans="2:16" ht="47.25" thickBot="1" x14ac:dyDescent="0.75">
       <c r="B2" s="2"/>
       <c r="C2" s="3" t="s">
         <v>3</v>
@@ -1008,8 +1010,9 @@
       <c r="L2" s="4"/>
       <c r="M2" s="4"/>
       <c r="N2" s="5"/>
+      <c r="O2" s="2"/>
     </row>
-    <row r="3" spans="2:16" ht="86.25" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:16" ht="186.75" thickBot="1" x14ac:dyDescent="0.75">
       <c r="B3" s="2"/>
       <c r="C3" s="6" t="s">
         <v>1</v>
@@ -1047,8 +1050,9 @@
       <c r="N3" s="8" t="s">
         <v>20</v>
       </c>
+      <c r="O3" s="2"/>
     </row>
-    <row r="4" spans="2:16" ht="29.25" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="4" spans="2:16" ht="47.25" thickBot="1" x14ac:dyDescent="0.75">
       <c r="B4" s="10" t="s">
         <v>22</v>
       </c>
@@ -1100,8 +1104,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="O4" s="2"/>
     </row>
-    <row r="5" spans="2:16" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:16" ht="46.5" x14ac:dyDescent="0.7">
       <c r="B5" s="15" t="s">
         <v>11</v>
       </c>
@@ -1131,8 +1136,9 @@
         <v>1</v>
       </c>
       <c r="N5" s="18"/>
+      <c r="O5" s="2"/>
     </row>
-    <row r="6" spans="2:16" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:16" ht="46.5" x14ac:dyDescent="0.7">
       <c r="B6" s="20" t="s">
         <v>12</v>
       </c>
@@ -1162,8 +1168,9 @@
         <v>1</v>
       </c>
       <c r="N6" s="23"/>
+      <c r="O6" s="2"/>
     </row>
-    <row r="7" spans="2:16" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:16" ht="46.5" x14ac:dyDescent="0.7">
       <c r="B7" s="20" t="s">
         <v>13</v>
       </c>
@@ -1191,8 +1198,9 @@
         <v>1</v>
       </c>
       <c r="N7" s="23"/>
+      <c r="O7" s="2"/>
     </row>
-    <row r="8" spans="2:16" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:16" ht="46.5" x14ac:dyDescent="0.7">
       <c r="B8" s="20" t="s">
         <v>14</v>
       </c>
@@ -1226,8 +1234,9 @@
         <v>1</v>
       </c>
       <c r="N8" s="23"/>
+      <c r="O8" s="2"/>
     </row>
-    <row r="9" spans="2:16" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:16" ht="46.5" x14ac:dyDescent="0.7">
       <c r="B9" s="20" t="s">
         <v>15</v>
       </c>
@@ -1257,11 +1266,12 @@
       </c>
       <c r="M9" s="24"/>
       <c r="N9" s="23"/>
+      <c r="O9" s="2"/>
       <c r="P9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="2:16" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:16" ht="47.25" thickBot="1" x14ac:dyDescent="0.75">
       <c r="B10" s="25" t="s">
         <v>16</v>
       </c>
@@ -1279,8 +1289,9 @@
       <c r="L10" s="27"/>
       <c r="M10" s="30"/>
       <c r="N10" s="28"/>
+      <c r="O10" s="2"/>
     </row>
-    <row r="11" spans="2:16" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:16" ht="46.5" x14ac:dyDescent="0.7">
       <c r="B11" s="31" t="s">
         <v>23</v>
       </c>
@@ -1311,8 +1322,9 @@
       <c r="L11" s="33"/>
       <c r="M11" s="33"/>
       <c r="N11" s="34"/>
+      <c r="O11" s="2"/>
     </row>
-    <row r="12" spans="2:16" ht="29.25" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="12" spans="2:16" ht="47.25" thickBot="1" x14ac:dyDescent="0.75">
       <c r="B12" s="38" t="s">
         <v>21</v>
       </c>
@@ -1338,8 +1350,40 @@
       <c r="L12" s="40"/>
       <c r="M12" s="40"/>
       <c r="N12" s="41"/>
+      <c r="O12" s="2"/>
     </row>
-    <row r="13" spans="2:16" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="2:16" s="1" customFormat="1" ht="46.5" x14ac:dyDescent="0.7">
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
+      <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
+      <c r="N13" s="2"/>
+      <c r="O13" s="2"/>
+    </row>
+    <row r="14" spans="2:16" ht="46.5" x14ac:dyDescent="0.7">
+      <c r="B14" s="45"/>
+      <c r="C14" s="45"/>
+      <c r="D14" s="45"/>
+      <c r="E14" s="45"/>
+      <c r="F14" s="45"/>
+      <c r="G14" s="45"/>
+      <c r="H14" s="45"/>
+      <c r="I14" s="45"/>
+      <c r="J14" s="45"/>
+      <c r="K14" s="45"/>
+      <c r="L14" s="45"/>
+      <c r="M14" s="45"/>
+      <c r="N14" s="45"/>
+      <c r="O14" s="2"/>
+    </row>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="C2:E2"/>

</xml_diff>